<commit_message>
Add SafetyOps Copilot and Analytics Copilot (Text-to-SQL) projects
Both lead Selected Work with live demo + repo links. Adds fine-tuning,
event-driven, and CV skills to the stack; updates marquee keywords and
the shipped-tests stat to span four systems.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/content.xlsx
+++ b/content/content.xlsx
@@ -568,10 +568,10 @@
         <v>Tests Across Shipped ML Systems</v>
       </c>
       <c r="B5" t="str">
-        <v>740+</v>
+        <v>810+</v>
       </c>
       <c r="C5" t="str">
-        <v>343 in the RAG backend + ~399 in the churn MLOps stack</v>
+        <v>Across four shipped ML systems — RAG backend, churn MLOps, Text-to-SQL, and SafetyOps</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -1003,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D73"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1915,9 +1915,121 @@
         <v>64</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Fine-Tuning (QLoRA · PEFT)</v>
+      </c>
+      <c r="B66" t="str">
+        <v>GenAI/NLP</v>
+      </c>
+      <c r="C66" t="str">
+        <v/>
+      </c>
+      <c r="D66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Unsloth</v>
+      </c>
+      <c r="B67" t="str">
+        <v>GenAI/NLP</v>
+      </c>
+      <c r="C67" t="str">
+        <v/>
+      </c>
+      <c r="D67">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Text-to-SQL</v>
+      </c>
+      <c r="B68" t="str">
+        <v>GenAI/NLP</v>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>YOLOv8</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Deep Learning</v>
+      </c>
+      <c r="C69" t="str">
+        <v/>
+      </c>
+      <c r="D69">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>DistilBERT</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Deep Learning</v>
+      </c>
+      <c r="C70" t="str">
+        <v/>
+      </c>
+      <c r="D70">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Redis Streams</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Data Engineering</v>
+      </c>
+      <c r="C71" t="str">
+        <v/>
+      </c>
+      <c r="D71">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Grafana</v>
+      </c>
+      <c r="B72" t="str">
+        <v>DevOps</v>
+      </c>
+      <c r="C72" t="str">
+        <v/>
+      </c>
+      <c r="D72">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>PostgreSQL</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Data</v>
+      </c>
+      <c r="C73" t="str">
+        <v/>
+      </c>
+      <c r="D73">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D73"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1960,7 +2072,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>LangGraph</v>
+        <v>LLM Fine-Tuning</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1968,7 +2080,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Python</v>
+        <v>LangGraph</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1976,7 +2088,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SQL</v>
+        <v>Python</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -1984,7 +2096,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PyTorch</v>
+        <v>SQL</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1992,7 +2104,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>XGBoost</v>
+        <v>PyTorch</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -2000,7 +2112,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MLflow</v>
+        <v>XGBoost</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -2008,7 +2120,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Docker</v>
+        <v>MLflow</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -2016,7 +2128,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>AWS SageMaker</v>
+        <v>Docker</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -2024,7 +2136,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>FastAPI</v>
+        <v>AWS SageMaker</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -2032,7 +2144,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Pinecone</v>
+        <v>FastAPI</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -2040,7 +2152,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SHAP</v>
+        <v>Event-Driven Systems</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -2048,7 +2160,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Streamlit</v>
+        <v>SHAP</v>
       </c>
       <c r="B16">
         <v>15</v>
@@ -2189,7 +2301,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2237,34 +2349,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>proj-rag-workbench</v>
+        <v>proj-safetyops-copilot</v>
       </c>
       <c r="B2" t="str">
-        <v>RAG Agent Workbench</v>
+        <v>SafetyOps Copilot</v>
       </c>
       <c r="C2" t="str">
-        <v>Agentic RAG backend: 8-node LangGraph pipeline with corrective retrieval, faithfulness verification, and SSE streaming.</v>
+        <v>Event-driven safety-incident platform: Redis Streams pipeline, DistilBERT severity scoring on 273k real MSHA narratives, YOLOv8 PPE detection, and a LangGraph triage copilot.</v>
       </c>
       <c r="D2" t="str">
-        <v>A production retrieval-augmented generation backend built as an 8-node LangGraph pipeline with conditional routing: query normalization → multi-turn contextualization → dense retrieval (Pinecone, llama-text-embed-v2) → bounded corrective retrieval (CRAG) → web-fallback routing (Tavily) → grounded generation (Groq Llama 3.1) → faithfulness verification. A deterministic retrieval-evaluation harness (recall@k, MRR, nDCG@k over a hand-labeled golden set) drove real decisions — including measuring a hosted reranker net-negative (nDCG@3 −0.057, +435 ms) and disabling it on the data.</v>
+        <v>An event-driven incident monitoring platform for industrial EHS teams, built as three independently deployable services (FastAPI API, Streamlit UI, background worker) connected by a Redis Streams message bus over shared Postgres. Free-text reports are scored for severity by a DistilBERT model fine-tuned on 273,000 real MSHA accident narratives (labels derived from regulatory outcome codes, not synthetic data), site photos are scored for PPE compliance by YOLOv8n, and a 5-node LangGraph state machine generates structured triage briefs — deterministic and fully testable without any LLM, with the LLM as an optional enhancement layer that fails silently back to the deterministic draft.</v>
       </c>
       <c r="E2" t="str">
-        <v>GenAI;RAG;LangGraph;LLM;Agentic AI;NLP</v>
+        <v>MLOps;Event-Driven Architecture;Computer Vision;NLP;LangGraph;Production ML</v>
       </c>
       <c r="F2" t="str">
-        <v>Python;FastAPI;LangGraph;Pinecone;Groq;Tavily;Prometheus;Docker;Hugging Face Spaces;Streamlit</v>
+        <v>Python;FastAPI;Redis Streams;PostgreSQL;SQLAlchemy;LangGraph;DistilBERT;YOLOv8;Docker;Prometheus;Grafana;Evidently;MLflow;DVC;Streamlit</v>
       </c>
       <c r="G2" t="str">
-        <v>https://github.com/brej-29/rag-agent-workbench</v>
+        <v>https://github.com/brej-29/safetyops-copilot</v>
       </c>
       <c r="H2" t="str">
-        <v>https://rag-agent-workbench.streamlit.app/</v>
+        <v>https://safetyops-copilot.streamlit.app/</v>
       </c>
       <c r="I2" t="str">
-        <v>8-node agentic LangGraph pipeline with conditional routing and bounded CRAG loop (provably non-runaway iteration cap);Deterministic retrieval-eval harness (recall@k, MRR, nDCG@k) on a hand-labeled golden set — used to A/B-test and reject a hosted reranker on data;Two-threshold retrieval gate with deterministic abstention (the LLM is never asked to answer from empty context) + indirect prompt-injection hardening;Per-request token/cost accounting, Prometheus latency histograms, true SSE token streaming;343 tests, CI from a hash-pinned lockfile; deployed on Docker / Hugging Face Spaces + Streamlit Cloud</v>
+        <v>DistilBERT severity classifier trained on 273k real MSHA narratives — 0.78 macro-F1 vs 0.34 rule-based baseline (95% relative lift) and 0.88 high-severity recall (5.5x the baseline);YOLOv8n PPE compliance detection (mAP@0.5 ≈ 0.81) behind a wrapper normalizing three different label-scheme conventions into one score;Redis Streams consumer groups with 3x exponential-backoff retry, dead-letter queue with replay, and idempotent processing keyed on stream message ID — safe under worker crash-restarts;Graceful ML degradation: both models sit behind lazy imports so the full pipeline, tests, and CI run with zero ML dependencies installed — 36 tests pass without torch;Evidently drift reports, Prometheus metrics on API and worker, and an 8-panel Grafana dashboard; ~5,100 LOC across 124 files</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-05</v>
+        <v>2026-07</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -2272,43 +2384,37 @@
       <c r="L2" t="str">
         <v/>
       </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>proj-dogbreed-classification</v>
+        <v>proj-analytics-copilot</v>
       </c>
       <c r="B3" t="str">
-        <v>Dog Breed Classification</v>
+        <v>Analytics Copilot (Text-to-SQL)</v>
       </c>
       <c r="C3" t="str">
-        <v>Deep learning pipeline for 120-breed classification with transfer learning.</v>
+        <v>Mistral-7B fine-tuned with QLoRA to turn natural language into schema-conditioned SQL, with a from-scratch evaluation harness and dual-provider inference failover.</v>
       </c>
       <c r="D3" t="str">
-        <v>End-to-end deep learning solution leveraging MobileNetV2 transfer learning to classify 120 dog breeds with optimized accuracy. Demonstrates proficiency in computer vision, data preprocessing, and model architecture selection—key skills for ML production environments.</v>
+        <v>A full fine-tuning pipeline — dataset curation, QLoRA training, custom dual-benchmark evaluation, Hub publishing — wrapped in a production-shaped serving layer. Mistral-7B-Instruct is fine-tuned with 4-bit NF4 quantization and LoRA adapters (r=16) across all seven attention and MLP projections, then served through a Hugging Face Inference Endpoint with adapter routing and an OpenAI fallback. The Streamlit front end carries zero GPU or ML runtime dependencies: training and serving are fully decoupled.</v>
       </c>
       <c r="E3" t="str">
-        <v>TensorFlow;Transfer Learning;CNN;Computer Vision</v>
+        <v>GenAI;LLM Fine-Tuning;QLoRA;Text-to-SQL;NLP;Model Evaluation</v>
       </c>
       <c r="F3" t="str">
-        <v>Python;TensorFlow;Jupyter</v>
+        <v>Python;Mistral-7B;QLoRA;PEFT;Unsloth;TRL;bitsandbytes;Transformers;sqlglot;Hugging Face Endpoints;Streamlit;GitHub Actions</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>https://github.com/brej-29/analytics-copilot-text2sql</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>https://analytics-copilot-text2sql.streamlit.app/</v>
       </c>
       <c r="I3" t="str">
-        <v>Transfer learning optimization;120-class multi-label classification;Production-ready preprocessing pipeline</v>
+        <v>Fine-tuned a 7B model with under 1% trainable parameters via 4-bit NF4 quantization and LoRA r=16 adapters across seven projection matrices;Built a from-scratch evaluation harness — Exact Match, literal-masked structural EM, sqlglot parse-validity, and AST-based schema-adherence checking that catches hallucinated tables and columns string similarity would miss;Dual-benchmark evaluation quantifying the generalization gap: 35.0% exact match / 100% parse success / 97.5% schema adherence in-domain, vs 76% schema adherence zero-shot on Spider;Multi-tier inference failover (HF Inference Endpoint with adapter routing → OpenAI) plus a proactive endpoint wake-up ping, deliberately separated so warm-ups never trigger the failure path;Root-caused a 271-violation CI lint break as upstream linter drift rather than new code, fixing it with a 9-line config pin instead of a repo-wide reformat; ~6,419 LOC, 36 tests across 14 files</v>
       </c>
       <c r="J3" t="str">
-        <v>2025-11</v>
+        <v>2026-06</v>
       </c>
       <c r="K3">
         <v>2</v>
@@ -2316,43 +2422,37 @@
       <c r="L3" t="str">
         <v/>
       </c>
-      <c r="M3" t="str">
-        <v>https://github.com/brej-29/Logicmojo-AIML-Assignments-DogBreedClassificationTensorFlow</v>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>proj-heart-disease</v>
+        <v>proj-rag-workbench</v>
       </c>
       <c r="B4" t="str">
-        <v>Heart Disease Risk Predictor</v>
+        <v>RAG Agent Workbench</v>
       </c>
       <c r="C4" t="str">
-        <v>Predictive model for cardiac disease classification from medical data.</v>
+        <v>Agentic RAG backend: 8-node LangGraph pipeline with corrective retrieval, faithfulness verification, and SSE streaming.</v>
       </c>
       <c r="D4" t="str">
-        <v>Comprehensive supervised learning pipeline for predicting heart disease risk using patient medical records. Features rigorous data exploration, model selection across multiple algorithms, hyperparameter tuning, and cross-validation—demonstrating systematic ML workflow and healthcare domain understanding.</v>
+        <v>A production retrieval-augmented generation backend built as an 8-node LangGraph pipeline with conditional routing: query normalization → multi-turn contextualization → dense retrieval (Pinecone, llama-text-embed-v2) → bounded corrective retrieval (CRAG) → web-fallback routing (Tavily) → grounded generation (Groq Llama 3.1) → faithfulness verification. A deterministic retrieval-evaluation harness (recall@k, MRR, nDCG@k over a hand-labeled golden set) drove real decisions — including measuring a hosted reranker net-negative (nDCG@3 −0.057, +435 ms) and disabling it on the data.</v>
       </c>
       <c r="E4" t="str">
-        <v>Machine Learning;Classification;Healthcare Analytics;Feature Engineering</v>
+        <v>GenAI;RAG;LangGraph;LLM;Agentic AI;NLP</v>
       </c>
       <c r="F4" t="str">
-        <v>Python;Scikit-learn;Pandas;Numpy</v>
+        <v>Python;FastAPI;LangGraph;Pinecone;Groq;Tavily;Prometheus;Docker;Hugging Face Spaces;Streamlit</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>https://github.com/brej-29/rag-agent-workbench</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>https://rag-agent-workbench.streamlit.app/</v>
       </c>
       <c r="I4" t="str">
-        <v>Multi-algorithm comparison;Cross-validated evaluation;Medical data preprocessing</v>
+        <v>8-node agentic LangGraph pipeline with conditional routing and bounded CRAG loop (provably non-runaway iteration cap);Deterministic retrieval-eval harness (recall@k, MRR, nDCG@k) on a hand-labeled golden set — used to A/B-test and reject a hosted reranker on data;Two-threshold retrieval gate with deterministic abstention (the LLM is never asked to answer from empty context) + indirect prompt-injection hardening;Per-request token/cost accounting, Prometheus latency histograms, true SSE token streaming;343 tests, CI from a hash-pinned lockfile; deployed on Docker / Hugging Face Spaces + Streamlit Cloud</v>
       </c>
       <c r="J4" t="str">
-        <v>2025-10</v>
+        <v>2026-05</v>
       </c>
       <c r="K4">
         <v>3</v>
@@ -2361,7 +2461,7 @@
         <v/>
       </c>
       <c r="M4" t="str">
-        <v>https://github.com/brej-29/Logicmojo-AIML-Assignments-heart-disease-prediction-ml</v>
+        <v/>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -2369,22 +2469,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>proj-bulldozer-price</v>
+        <v>proj-dogbreed-classification</v>
       </c>
       <c r="B5" t="str">
-        <v>Heavy Equipment Price Prediction</v>
+        <v>Dog Breed Classification</v>
       </c>
       <c r="C5" t="str">
-        <v>Regression model for predicting equipment resale values.</v>
+        <v>Deep learning pipeline for 120-breed classification with transfer learning.</v>
       </c>
       <c r="D5" t="str">
-        <v>Full-stack data science project predicting bulldozer auction prices using real-world commodity data. Covers complete pipeline: feature engineering, handling temporal data, model ensembling with XGBoost, and RMSLE optimization. Demonstrates end-to-end problem-solving from raw data to production predictions.</v>
+        <v>End-to-end deep learning solution leveraging MobileNetV2 transfer learning to classify 120 dog breeds with optimized accuracy. Demonstrates proficiency in computer vision, data preprocessing, and model architecture selection—key skills for ML production environments.</v>
       </c>
       <c r="E5" t="str">
-        <v>Regression;XGBoost;Ensemble Methods;Time-Series Features</v>
+        <v>TensorFlow;Transfer Learning;CNN;Computer Vision</v>
       </c>
       <c r="F5" t="str">
-        <v>Python;XGBoost;Scikit-learn;Pandas</v>
+        <v>Python;TensorFlow;Jupyter</v>
       </c>
       <c r="G5" t="str">
         <v/>
@@ -2393,10 +2493,10 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>XGBoost ensembling;Feature engineering for auction data;RMSLE optimization;Real-world dataset handling</v>
+        <v>Transfer learning optimization;120-class multi-label classification;Production-ready preprocessing pipeline</v>
       </c>
       <c r="J5" t="str">
-        <v>2025-09</v>
+        <v>2025-11</v>
       </c>
       <c r="K5">
         <v>4</v>
@@ -2405,7 +2505,7 @@
         <v/>
       </c>
       <c r="M5" t="str">
-        <v>https://github.com/brej-29/Logicmojo-AIML-Assignments-bulldozer-price-prediction</v>
+        <v>https://github.com/brej-29/Logicmojo-AIML-Assignments-DogBreedClassificationTensorFlow</v>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -2413,22 +2513,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>proj-otaku-oracle</v>
+        <v>proj-heart-disease</v>
       </c>
       <c r="B6" t="str">
-        <v>Otaku Oracle</v>
+        <v>Heart Disease Risk Predictor</v>
       </c>
       <c r="C6" t="str">
-        <v>Intelligent anime recommendation engine powered by NLP.</v>
+        <v>Predictive model for cardiac disease classification from medical data.</v>
       </c>
       <c r="D6" t="str">
-        <v>AI-driven recommendation system applying NLP and collaborative filtering to anime datasets. Demonstrates understanding of recommendation systems, text processing, and user preference modeling—critical for personalization in production ML systems.</v>
+        <v>Comprehensive supervised learning pipeline for predicting heart disease risk using patient medical records. Features rigorous data exploration, model selection across multiple algorithms, hyperparameter tuning, and cross-validation—demonstrating systematic ML workflow and healthcare domain understanding.</v>
       </c>
       <c r="E6" t="str">
-        <v>NLP;Recommendation Systems;Collaborative Filtering</v>
+        <v>Machine Learning;Classification;Healthcare Analytics;Feature Engineering</v>
       </c>
       <c r="F6" t="str">
-        <v>Python;NLTK;Scikit-learn</v>
+        <v>Python;Scikit-learn;Pandas;Numpy</v>
       </c>
       <c r="G6" t="str">
         <v/>
@@ -2437,10 +2537,10 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>Custom recommendation algorithm;NLP-based feature extraction;Cold-start problem handling</v>
+        <v>Multi-algorithm comparison;Cross-validated evaluation;Medical data preprocessing</v>
       </c>
       <c r="J6" t="str">
-        <v>2025-08</v>
+        <v>2025-10</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -2449,7 +2549,7 @@
         <v/>
       </c>
       <c r="M6" t="str">
-        <v>https://github.com/brej-29/otaku-oracle</v>
+        <v>https://github.com/brej-29/Logicmojo-AIML-Assignments-heart-disease-prediction-ml</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -2457,22 +2557,22 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>proj-meal-planner</v>
+        <v>proj-bulldozer-price</v>
       </c>
       <c r="B7" t="str">
-        <v>Daily Meal Planner</v>
+        <v>Heavy Equipment Price Prediction</v>
       </c>
       <c r="C7" t="str">
-        <v>Personalized nutrition planning with Streamlit interface.</v>
+        <v>Regression model for predicting equipment resale values.</v>
       </c>
       <c r="D7" t="str">
-        <v>Interactive Streamlit application generating daily meal plans based on nutritional goals and dietary constraints. Showcases full-stack ML application development: requirement gathering, algorithm design, and user-centric UI/UX implementation.</v>
+        <v>Full-stack data science project predicting bulldozer auction prices using real-world commodity data. Covers complete pipeline: feature engineering, handling temporal data, model ensembling with XGBoost, and RMSLE optimization. Demonstrates end-to-end problem-solving from raw data to production predictions.</v>
       </c>
       <c r="E7" t="str">
-        <v>Streamlit;Nutrition Algorithm;API Integration</v>
+        <v>Regression;XGBoost;Ensemble Methods;Time-Series Features</v>
       </c>
       <c r="F7" t="str">
-        <v>Python;Streamlit;APIs</v>
+        <v>Python;XGBoost;Scikit-learn;Pandas</v>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -2481,10 +2581,10 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>Intelligent constraint solver;Real-time API data;Production Streamlit deployment</v>
+        <v>XGBoost ensembling;Feature engineering for auction data;RMSLE optimization;Real-world dataset handling</v>
       </c>
       <c r="J7" t="str">
-        <v>2025-07</v>
+        <v>2025-09</v>
       </c>
       <c r="K7">
         <v>6</v>
@@ -2493,30 +2593,30 @@
         <v/>
       </c>
       <c r="M7" t="str">
-        <v>https://github.com/brej-29/daily-meal-planner-streamlit</v>
+        <v>https://github.com/brej-29/Logicmojo-AIML-Assignments-bulldozer-price-prediction</v>
       </c>
       <c r="N7" t="str">
-        <v>https://daily-meal-planner.streamlit.app/</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>proj-workout-planner</v>
+        <v>proj-otaku-oracle</v>
       </c>
       <c r="B8" t="str">
-        <v>Daily Workout Planner</v>
+        <v>Otaku Oracle</v>
       </c>
       <c r="C8" t="str">
-        <v>ML-powered fitness program generator.</v>
+        <v>Intelligent anime recommendation engine powered by NLP.</v>
       </c>
       <c r="D8" t="str">
-        <v>Smart workout recommendation engine tailored to user fitness levels, goals, and equipment availability. Demonstrates machine learning application in domain-specific personalization and real-time system adaptability.</v>
+        <v>AI-driven recommendation system applying NLP and collaborative filtering to anime datasets. Demonstrates understanding of recommendation systems, text processing, and user preference modeling—critical for personalization in production ML systems.</v>
       </c>
       <c r="E8" t="str">
-        <v>Streamlit;Fitness Algorithm;Personalization</v>
+        <v>NLP;Recommendation Systems;Collaborative Filtering</v>
       </c>
       <c r="F8" t="str">
-        <v>Python;Streamlit;Pandas</v>
+        <v>Python;NLTK;Scikit-learn</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -2525,10 +2625,10 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>Progressive workout scaling;Goal-oriented recommendations;Equipment constraint handling</v>
+        <v>Custom recommendation algorithm;NLP-based feature extraction;Cold-start problem handling</v>
       </c>
       <c r="J8" t="str">
-        <v>2025-06</v>
+        <v>2025-08</v>
       </c>
       <c r="K8">
         <v>7</v>
@@ -2537,30 +2637,30 @@
         <v/>
       </c>
       <c r="M8" t="str">
-        <v>https://github.com/brej-29/daily-workout-planner</v>
+        <v>https://github.com/brej-29/otaku-oracle</v>
       </c>
       <c r="N8" t="str">
-        <v>https://brejesh-daily-workout-planner.streamlit.app/</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>proj-aurora-chat</v>
+        <v>proj-meal-planner</v>
       </c>
       <c r="B9" t="str">
-        <v>Aurora Chat</v>
+        <v>Daily Meal Planner</v>
       </c>
       <c r="C9" t="str">
-        <v>Real-time AI chatbot with LLM integration.</v>
+        <v>Personalized nutrition planning with Streamlit interface.</v>
       </c>
       <c r="D9" t="str">
-        <v>Production-grade conversational AI application leveraging LLMs for natural dialogue. Demonstrates prompt engineering, context management, and real-time inference optimization—essential for modern ML applications in NLP.</v>
+        <v>Interactive Streamlit application generating daily meal plans based on nutritional goals and dietary constraints. Showcases full-stack ML application development: requirement gathering, algorithm design, and user-centric UI/UX implementation.</v>
       </c>
       <c r="E9" t="str">
-        <v>LLM;NLP;Chatbot;Prompt Engineering</v>
+        <v>Streamlit;Nutrition Algorithm;API Integration</v>
       </c>
       <c r="F9" t="str">
-        <v>Python;Streamlit;LangChain;OpenAI API</v>
+        <v>Python;Streamlit;APIs</v>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -2569,10 +2669,10 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>LLM prompt optimization;Token-efficient context handling;Real-time streaming responses</v>
+        <v>Intelligent constraint solver;Real-time API data;Production Streamlit deployment</v>
       </c>
       <c r="J9" t="str">
-        <v>2025-05</v>
+        <v>2025-07</v>
       </c>
       <c r="K9">
         <v>8</v>
@@ -2581,30 +2681,30 @@
         <v/>
       </c>
       <c r="M9" t="str">
-        <v>https://github.com/brej-29/aurora-chat-streamlit</v>
+        <v>https://github.com/brej-29/daily-meal-planner-streamlit</v>
       </c>
       <c r="N9" t="str">
-        <v>https://aurora-chat.streamlit.app/</v>
+        <v>https://daily-meal-planner.streamlit.app/</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>proj-hr-analytics</v>
+        <v>proj-workout-planner</v>
       </c>
       <c r="B10" t="str">
-        <v>HR Analytics Dashboard</v>
+        <v>Daily Workout Planner</v>
       </c>
       <c r="C10" t="str">
-        <v>Workforce intelligence platform with Power BI.</v>
+        <v>ML-powered fitness program generator.</v>
       </c>
       <c r="D10" t="str">
-        <v>Comprehensive business analytics dashboard analyzing HR metrics, employee performance, and organizational trends. Demonstrates data visualization expertise, business intelligence fundamentals, and ability to translate data insights into actionable business metrics.</v>
+        <v>Smart workout recommendation engine tailored to user fitness levels, goals, and equipment availability. Demonstrates machine learning application in domain-specific personalization and real-time system adaptability.</v>
       </c>
       <c r="E10" t="str">
-        <v>Power BI;Business Analytics;Data Visualization;KPI Tracking</v>
+        <v>Streamlit;Fitness Algorithm;Personalization</v>
       </c>
       <c r="F10" t="str">
-        <v>Power BI;SQL;Excel</v>
+        <v>Python;Streamlit;Pandas</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -2613,10 +2713,10 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>Interactive KPI dashboards;Employee retention analytics;Drill-down analytics</v>
+        <v>Progressive workout scaling;Goal-oriented recommendations;Equipment constraint handling</v>
       </c>
       <c r="J10" t="str">
-        <v>2025-04</v>
+        <v>2025-06</v>
       </c>
       <c r="K10">
         <v>9</v>
@@ -2625,30 +2725,30 @@
         <v/>
       </c>
       <c r="M10" t="str">
-        <v>https://github.com/brej-29/hr-analytics-dashboard-powerbi</v>
+        <v>https://github.com/brej-29/daily-workout-planner</v>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>https://brejesh-daily-workout-planner.streamlit.app/</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>proj-essay-writer</v>
+        <v>proj-aurora-chat</v>
       </c>
       <c r="B11" t="str">
-        <v>Essay Writer</v>
+        <v>Aurora Chat</v>
       </c>
       <c r="C11" t="str">
-        <v>Intelligent essay generation with structured outputs.</v>
+        <v>Real-time AI chatbot with LLM integration.</v>
       </c>
       <c r="D11" t="str">
-        <v>LLM-powered content generation system producing well-structured essays with customizable prompts and export functionality. Demonstrates prompt tuning, output formatting, and practical application of language models for content generation.</v>
+        <v>Production-grade conversational AI application leveraging LLMs for natural dialogue. Demonstrates prompt engineering, context management, and real-time inference optimization—essential for modern ML applications in NLP.</v>
       </c>
       <c r="E11" t="str">
-        <v>LLM;NLP;Content Generation;Prompt Engineering</v>
+        <v>LLM;NLP;Chatbot;Prompt Engineering</v>
       </c>
       <c r="F11" t="str">
-        <v>Python;Streamlit;LangChain</v>
+        <v>Python;Streamlit;LangChain;OpenAI API</v>
       </c>
       <c r="G11" t="str">
         <v/>
@@ -2657,10 +2757,10 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>Structured prompt templates;Multi-format export;Iterative refinement capability</v>
+        <v>LLM prompt optimization;Token-efficient context handling;Real-time streaming responses</v>
       </c>
       <c r="J11" t="str">
-        <v>2025-03</v>
+        <v>2025-05</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -2669,30 +2769,30 @@
         <v/>
       </c>
       <c r="M11" t="str">
-        <v>https://github.com/brej-29/essay-writer-streamlit</v>
+        <v>https://github.com/brej-29/aurora-chat-streamlit</v>
       </c>
       <c r="N11" t="str">
-        <v>https://essay-writer-app.streamlit.app/</v>
+        <v>https://aurora-chat.streamlit.app/</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>proj-disaster-nlp</v>
+        <v>proj-hr-analytics</v>
       </c>
       <c r="B12" t="str">
-        <v>Disaster Tweets — NLP Architecture Benchmarks</v>
+        <v>HR Analytics Dashboard</v>
       </c>
       <c r="C12" t="str">
-        <v>7 architectures benchmarked on ~7,600 tweets — USE transfer learning wins at 81.5% accuracy / 0.81 F1.</v>
+        <v>Workforce intelligence platform with Power BI.</v>
       </c>
       <c r="D12" t="str">
-        <v>A controlled NLP benchmarking study across 7 architectures — TF-IDF + Naive Bayes, Dense, LSTM, GRU, BiLSTM, Conv1D, and Universal Sentence Encoder transfer learning — on ~7,600 disaster tweets with a consistent 90/10 split. USE transfer learning achieved the best results (81.5% accuracy, 0.81 F1), demonstrating that pre-trained encoders outperform from-scratch models on small datasets.</v>
+        <v>Comprehensive business analytics dashboard analyzing HR metrics, employee performance, and organizational trends. Demonstrates data visualization expertise, business intelligence fundamentals, and ability to translate data insights into actionable business metrics.</v>
       </c>
       <c r="E12" t="str">
-        <v>NLP;Deep Learning;Transfer Learning;Model Benchmarking;TensorFlow</v>
+        <v>Power BI;Business Analytics;Data Visualization;KPI Tracking</v>
       </c>
       <c r="F12" t="str">
-        <v>Python;TensorFlow;TensorFlow Hub;scikit-learn;Pandas</v>
+        <v>Power BI;SQL;Excel</v>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -2701,10 +2801,10 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>7 architectures under identical splits: classical ML, RNN family (LSTM/GRU/BiLSTM), Conv1D, and USE transfer learning;Best model: Universal Sentence Encoder transfer learning — 81.5% accuracy, 0.81 F1;Clear evidence that pre-trained encoders beat from-scratch models on small text datasets</v>
+        <v>Interactive KPI dashboards;Employee retention analytics;Drill-down analytics</v>
       </c>
       <c r="J12" t="str">
-        <v>2025-02</v>
+        <v>2025-04</v>
       </c>
       <c r="K12">
         <v>11</v>
@@ -2713,7 +2813,7 @@
         <v/>
       </c>
       <c r="M12" t="str">
-        <v>https://github.com/brej-29/disaster-tweets-nlp-model-benchmarks</v>
+        <v>https://github.com/brej-29/hr-analytics-dashboard-powerbi</v>
       </c>
       <c r="N12" t="str">
         <v/>
@@ -2721,22 +2821,22 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>proj-inventory-classifier</v>
+        <v>proj-essay-writer</v>
       </c>
       <c r="B13" t="str">
-        <v>Inventory Bin Classification — CV on SageMaker</v>
+        <v>Essay Writer</v>
       </c>
       <c r="C13" t="str">
-        <v>ResNet-50 transfer learning on 10,000+ warehouse images with SageMaker Bayesian HPO, distributed spot training, and a live endpoint.</v>
+        <v>Intelligent essay generation with structured outputs.</v>
       </c>
       <c r="D13" t="str">
-        <v>An end-to-end computer vision pipeline classifying warehouse bin item counts from 10,000+ images using ResNet-50 transfer learning, with deterministic stratified splits stored as S3 ImageFolder channels. SageMaker Bayesian hyperparameter tuning (learning rate, weight decay, batch size, backbone-freeze) with 2-instance distributed training on managed spot instances delivered a ~22% macro-F1 gain over baseline. Served through a real-time SageMaker endpoint with a custom PyTorch inference handler and AWS Lambda integration.</v>
+        <v>LLM-powered content generation system producing well-structured essays with customizable prompts and export functionality. Demonstrates prompt tuning, output formatting, and practical application of language models for content generation.</v>
       </c>
       <c r="E13" t="str">
-        <v>Computer Vision;AWS SageMaker;MLOps;Deep Learning;Cloud Deployment</v>
+        <v>LLM;NLP;Content Generation;Prompt Engineering</v>
       </c>
       <c r="F13" t="str">
-        <v>Python;PyTorch;ResNet-50;AWS SageMaker;AWS Lambda;AWS S3;Docker</v>
+        <v>Python;Streamlit;LangChain</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -2745,10 +2845,10 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>~22% macro-F1 gain from SageMaker Bayesian HPO with 2-instance distributed training on managed spot instances;Deterministic stratified splits as S3 ImageFolder channels for reproducible training;Real-time SageMaker endpoint with custom PyTorch inference handler + Lambda (image URL / S3 URI → JSON label, confidence, probabilities);Full resource cleanup — no orphaned endpoints or storage</v>
+        <v>Structured prompt templates;Multi-format export;Iterative refinement capability</v>
       </c>
       <c r="J13" t="str">
-        <v>2025-01</v>
+        <v>2025-03</v>
       </c>
       <c r="K13">
         <v>12</v>
@@ -2757,30 +2857,30 @@
         <v/>
       </c>
       <c r="M13" t="str">
-        <v>https://github.com/brej-29/inventory-bin-count-classifier-aws-sagemaker</v>
+        <v>https://github.com/brej-29/essay-writer-streamlit</v>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>https://essay-writer-app.streamlit.app/</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>proj-aws-ml-nanodegree</v>
+        <v>proj-disaster-nlp</v>
       </c>
       <c r="B14" t="str">
-        <v>AWS ML Engineer Nanodegree</v>
+        <v>Disaster Tweets — NLP Architecture Benchmarks</v>
       </c>
       <c r="C14" t="str">
-        <v>Comprehensive AWS ML engineering curriculum projects.</v>
+        <v>7 architectures benchmarked on ~7,600 tweets — USE transfer learning wins at 81.5% accuracy / 0.81 F1.</v>
       </c>
       <c r="D14" t="str">
-        <v>Complete Udacity nanodegree covering AWS ML services, MLOps, and production ML pipelines. Includes projects on SageMaker, model deployment, monitoring, and hyperparameter optimization—essential competencies for ML engineering roles.</v>
+        <v>A controlled NLP benchmarking study across 7 architectures — TF-IDF + Naive Bayes, Dense, LSTM, GRU, BiLSTM, Conv1D, and Universal Sentence Encoder transfer learning — on ~7,600 disaster tweets with a consistent 90/10 split. USE transfer learning achieved the best results (81.5% accuracy, 0.81 F1), demonstrating that pre-trained encoders outperform from-scratch models on small datasets.</v>
       </c>
       <c r="E14" t="str">
-        <v>AWS;MLOps;SageMaker;ML Pipeline</v>
+        <v>NLP;Deep Learning;Transfer Learning;Model Benchmarking;TensorFlow</v>
       </c>
       <c r="F14" t="str">
-        <v>Python;AWS;Jupyter</v>
+        <v>Python;TensorFlow;TensorFlow Hub;scikit-learn;Pandas</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -2789,10 +2889,10 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>Hyperparameter optimization;Model monitoring;MLOps best practices;Automated pipelines</v>
+        <v>7 architectures under identical splits: classical ML, RNN family (LSTM/GRU/BiLSTM), Conv1D, and USE transfer learning;Best model: Universal Sentence Encoder transfer learning — 81.5% accuracy, 0.81 F1;Clear evidence that pre-trained encoders beat from-scratch models on small text datasets</v>
       </c>
       <c r="J14" t="str">
-        <v>2024-12</v>
+        <v>2025-02</v>
       </c>
       <c r="K14">
         <v>13</v>
@@ -2801,7 +2901,7 @@
         <v/>
       </c>
       <c r="M14" t="str">
-        <v>https://github.com/brej-29/udacity-AWS-ml-engineer-nanodegree</v>
+        <v>https://github.com/brej-29/disaster-tweets-nlp-model-benchmarks</v>
       </c>
       <c r="N14" t="str">
         <v/>
@@ -2809,34 +2909,34 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>proj-customer-churn</v>
+        <v>proj-inventory-classifier</v>
       </c>
       <c r="B15" t="str">
-        <v>Customer Churn Prediction — MLOps + GenAI</v>
+        <v>Inventory Bin Classification — CV on SageMaker</v>
       </c>
       <c r="C15" t="str">
-        <v>Leakage-safe churn model with Optuna-tuned XGBoost, SHAP-grounded LLM explanations, and a full MLOps loop — deployed live.</v>
+        <v>ResNet-50 transfer learning on 10,000+ warehouse images with SageMaker Bayesian HPO, distributed spot training, and a live endpoint.</v>
       </c>
       <c r="D15" t="str">
-        <v>End-to-end churn prediction on the IBM Telco dataset (7,043 records): six models benchmarked under 5-fold stratified CV on PR-AUC, XGBoost tuned with Optuna (PR-AUC 0.62→0.67) with isotonic calibration and a cost-based decision threshold from an explicit 5:1 FN:FP cost — test PR-AUC 0.66 / ROC-AUC 0.85 / recall 0.87. A SHAP-grounded LLM explanation layer feeds per-prediction drivers into Pydantic-validated explanations with RAG-retrieved retention tactics (sentence-transformers + FAISS); a two-tier faithfulness eval caught a real grounding bug and raised faithfulness 0.72→0.90.</v>
+        <v>An end-to-end computer vision pipeline classifying warehouse bin item counts from 10,000+ images using ResNet-50 transfer learning, with deterministic stratified splits stored as S3 ImageFolder channels. SageMaker Bayesian hyperparameter tuning (learning rate, weight decay, batch size, backbone-freeze) with 2-instance distributed training on managed spot instances delivered a ~22% macro-F1 gain over baseline. Served through a real-time SageMaker endpoint with a custom PyTorch inference handler and AWS Lambda integration.</v>
       </c>
       <c r="E15" t="str">
-        <v>MLOps;Machine Learning;GenAI;Explainability;Model Monitoring;XGBoost</v>
+        <v>Computer Vision;AWS SageMaker;MLOps;Deep Learning;Cloud Deployment</v>
       </c>
       <c r="F15" t="str">
-        <v>Python;XGBoost;Optuna;SHAP;MLflow;DVC;Pandera;Evidently;FastAPI;Docker;FAISS;GitHub Actions</v>
+        <v>Python;PyTorch;ResNet-50;AWS SageMaker;AWS Lambda;AWS S3;Docker</v>
       </c>
       <c r="G15" t="str">
         <v/>
       </c>
       <c r="H15" t="str">
-        <v>https://huggingface.co/spaces/BrejBala/churn-ui</v>
+        <v/>
       </c>
       <c r="I15" t="str">
-        <v>PR-AUC 0.62→0.67 via Optuna HPO; isotonic calibration + cost-based threshold (5:1 FN:FP); test ROC-AUC 0.85, recall 0.87;SHAP-grounded LLM explanations with RAG retention tactics; faithfulness eval raised 0.72→0.90 (n=50, seeded);Single-source Pandera data contract enforced across train and serve; Evidently drift monitoring with a 30%-drift retrain rule;MLflow champion/challenger registry on DagsHub with gated promotion; CI model-quality gate blocks merges below a PR-AUC floor;Docker image cut 57% (11.4→4.9 GB); deployed live to Hugging Face Spaces (FastAPI + Streamlit), ~399 tests</v>
+        <v>~22% macro-F1 gain from SageMaker Bayesian HPO with 2-instance distributed training on managed spot instances;Deterministic stratified splits as S3 ImageFolder channels for reproducible training;Real-time SageMaker endpoint with custom PyTorch inference handler + Lambda (image URL / S3 URI → JSON label, confidence, probabilities);Full resource cleanup — no orphaned endpoints or storage</v>
       </c>
       <c r="J15" t="str">
-        <v>2024-11</v>
+        <v>2025-01</v>
       </c>
       <c r="K15">
         <v>14</v>
@@ -2845,7 +2945,7 @@
         <v/>
       </c>
       <c r="M15" t="str">
-        <v>https://github.com/brej-29/customer-churn-mlops</v>
+        <v>https://github.com/brej-29/inventory-bin-count-classifier-aws-sagemaker</v>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -2853,22 +2953,22 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>proj-stock-terminal</v>
+        <v>proj-aws-ml-nanodegree</v>
       </c>
       <c r="B16" t="str">
-        <v>Stock Mini Terminal</v>
+        <v>AWS ML Engineer Nanodegree</v>
       </c>
       <c r="C16" t="str">
-        <v>Real-time stock analysis with fundamentals and technical indicators.</v>
+        <v>Comprehensive AWS ML engineering curriculum projects.</v>
       </c>
       <c r="D16" t="str">
-        <v>Production-grade financial analytics platform providing ticker search, price performance tracking, fundamental analysis, and news aggregation. Demonstrates proficiency in financial data processing, API integration, and building decision-support tools—valuable for data science roles in fintech and quantitative analysis.</v>
+        <v>Complete Udacity nanodegree covering AWS ML services, MLOps, and production ML pipelines. Includes projects on SageMaker, model deployment, monitoring, and hyperparameter optimization—essential competencies for ML engineering roles.</v>
       </c>
       <c r="E16" t="str">
-        <v>Streamlit;Financial Analytics;API Integration;Data Visualization</v>
+        <v>AWS;MLOps;SageMaker;ML Pipeline</v>
       </c>
       <c r="F16" t="str">
-        <v>Python;Streamlit;yfinance;APIs</v>
+        <v>Python;AWS;Jupyter</v>
       </c>
       <c r="G16" t="str">
         <v/>
@@ -2877,10 +2977,10 @@
         <v/>
       </c>
       <c r="I16" t="str">
-        <v>Real-time market data;Multi-source aggregation;Technical indicators dashboard</v>
+        <v>Hyperparameter optimization;Model monitoring;MLOps best practices;Automated pipelines</v>
       </c>
       <c r="J16" t="str">
-        <v>2025-12</v>
+        <v>2024-12</v>
       </c>
       <c r="K16">
         <v>15</v>
@@ -2889,42 +2989,42 @@
         <v/>
       </c>
       <c r="M16" t="str">
-        <v>https://github.com/brej-29/stock-mini-terminal-streamlit</v>
+        <v>https://github.com/brej-29/udacity-AWS-ml-engineer-nanodegree</v>
       </c>
       <c r="N16" t="str">
-        <v>https://stock-terminal.streamlit.app/</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>proj-data-insights-portal</v>
+        <v>proj-customer-churn</v>
       </c>
       <c r="B17" t="str">
-        <v>Collaborative Data Insights Portal</v>
+        <v>Customer Churn Prediction — MLOps + GenAI</v>
       </c>
       <c r="C17" t="str">
-        <v>Multi-user analytics platform for team-based data exploration.</v>
+        <v>Leakage-safe churn model with Optuna-tuned XGBoost, SHAP-grounded LLM explanations, and a full MLOps loop — deployed live.</v>
       </c>
       <c r="D17" t="str">
-        <v>Enterprise-level collaborative analytics application enabling teams to share datasets, generate insights, and visualize findings collectively. Showcases understanding of multi-user systems, data governance, and collaborative workflows—critical for data science teams in production environments.</v>
+        <v>End-to-end churn prediction on the IBM Telco dataset (7,043 records): six models benchmarked under 5-fold stratified CV on PR-AUC, XGBoost tuned with Optuna (PR-AUC 0.62→0.67) with isotonic calibration and a cost-based decision threshold from an explicit 5:1 FN:FP cost — test PR-AUC 0.66 / ROC-AUC 0.85 / recall 0.87. A SHAP-grounded LLM explanation layer feeds per-prediction drivers into Pydantic-validated explanations with RAG-retrieved retention tactics (sentence-transformers + FAISS); a two-tier faithfulness eval caught a real grounding bug and raised faithfulness 0.72→0.90.</v>
       </c>
       <c r="E17" t="str">
-        <v>Streamlit;Collaboration;Data Analytics;Dashboard</v>
+        <v>MLOps;Machine Learning;GenAI;Explainability;Model Monitoring;XGBoost</v>
       </c>
       <c r="F17" t="str">
-        <v>Python;Streamlit;Pandas;Plotly</v>
+        <v>Python;XGBoost;Optuna;SHAP;MLflow;DVC;Pandera;Evidently;FastAPI;Docker;FAISS;GitHub Actions</v>
       </c>
       <c r="G17" t="str">
         <v/>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>https://huggingface.co/spaces/BrejBala/churn-ui</v>
       </c>
       <c r="I17" t="str">
-        <v>Multi-user architecture;Shared dataset management;Interactive visualization;Role-based workflows</v>
+        <v>PR-AUC 0.62→0.67 via Optuna HPO; isotonic calibration + cost-based threshold (5:1 FN:FP); test ROC-AUC 0.85, recall 0.87;SHAP-grounded LLM explanations with RAG retention tactics; faithfulness eval raised 0.72→0.90 (n=50, seeded);Single-source Pandera data contract enforced across train and serve; Evidently drift monitoring with a 30%-drift retrain rule;MLflow champion/challenger registry on DagsHub with gated promotion; CI model-quality gate blocks merges below a PR-AUC floor;Docker image cut 57% (11.4→4.9 GB); deployed live to Hugging Face Spaces (FastAPI + Streamlit), ~399 tests</v>
       </c>
       <c r="J17" t="str">
-        <v>2025-11</v>
+        <v>2024-11</v>
       </c>
       <c r="K17">
         <v>16</v>
@@ -2933,15 +3033,103 @@
         <v/>
       </c>
       <c r="M17" t="str">
+        <v>https://github.com/brej-29/customer-churn-mlops</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>proj-stock-terminal</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Stock Mini Terminal</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Real-time stock analysis with fundamentals and technical indicators.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Production-grade financial analytics platform providing ticker search, price performance tracking, fundamental analysis, and news aggregation. Demonstrates proficiency in financial data processing, API integration, and building decision-support tools—valuable for data science roles in fintech and quantitative analysis.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Streamlit;Financial Analytics;API Integration;Data Visualization</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Python;Streamlit;yfinance;APIs</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v>Real-time market data;Multi-source aggregation;Technical indicators dashboard</v>
+      </c>
+      <c r="J18" t="str">
+        <v>2025-12</v>
+      </c>
+      <c r="K18">
+        <v>17</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v>https://github.com/brej-29/stock-mini-terminal-streamlit</v>
+      </c>
+      <c r="N18" t="str">
+        <v>https://stock-terminal.streamlit.app/</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>proj-data-insights-portal</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Collaborative Data Insights Portal</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Multi-user analytics platform for team-based data exploration.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Enterprise-level collaborative analytics application enabling teams to share datasets, generate insights, and visualize findings collectively. Showcases understanding of multi-user systems, data governance, and collaborative workflows—critical for data science teams in production environments.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Streamlit;Collaboration;Data Analytics;Dashboard</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Python;Streamlit;Pandas;Plotly</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>Multi-user architecture;Shared dataset management;Interactive visualization;Role-based workflows</v>
+      </c>
+      <c r="J19" t="str">
+        <v>2025-11</v>
+      </c>
+      <c r="K19">
+        <v>18</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
         <v>https://github.com/brej-29/collaborative-data-insights-portal</v>
       </c>
-      <c r="N17" t="str">
+      <c r="N19" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>